<commit_message>
E2E 92/110 after Quotes, Team Selling, Knowledge self-serve and handler fixes.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/AGENT LIBRARY/Reports/exports/GPTfy_Skill_Library_E2E.xlsx
+++ b/AGENT LIBRARY/Reports/exports/GPTfy_Skill_Library_E2E.xlsx
@@ -417,6 +417,10 @@
   </sheetPr>
   <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -434,7 +438,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-06 05:43 UTC</t>
+          <t>2026-08-06 07:32 UTC</t>
         </is>
       </c>
     </row>
@@ -482,7 +486,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>92</t>
         </is>
       </c>
     </row>
@@ -494,7 +498,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -518,7 +522,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -1003,7 +1007,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>fail_missing_feature</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1018,17 +1022,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>&lt;div&gt;⚠️ &lt;b&gt;Could not add team member&lt;/b&gt;&lt;br/&gt;OpportunityTeamMember is not creatable (Team Selling may be disabled).&lt;/div&gt;</t>
+          <t>{ "status": "Success", "message": "", "data": { "recordId": "00qQH000006mt0MYAQ", "message": "✅ Team Member Added Team role: Account Manager 👉 View Team Member", "success": true } }</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Feature / package not available in this org (expected N/A until enabled).</t>
+          <t>Skill executed successfully (Apex business success).</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Enable Team Selling (Setup → Opportunity Team Settings / Team Selling), ensure OpportunityTeamMember is creatable, then re-run.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1097,7 +1101,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>fail_data</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1107,22 +1111,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>{ "Quantity": 1, "UnitPrice": 10, "PricebookEntryId": "01uQH000003sGBCYA2" }</t>
+          <t>{ "QuoteId": "0Q0QH000002Bn7V0AS", "Quantity": 1, "UnitPrice": 10, "PricebookEntryId": "01uQH000003sGBCYA2" }</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>&lt;div&gt;⚠️ &lt;b&gt;Could not add quote line item&lt;/b&gt;&lt;br/&gt;Missing parameter: QuoteId&lt;/div&gt;</t>
+          <t>{ "status": "Success", "message": "", "data": { "recordId": "0QLQH000003nayH4AQ", "message": "✅ Quote Line Item Added Quantity: 1 Unit Price: 10 👉 View Line Item", "success": true } }</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Data / seed or missing parameter issue: &lt;div&gt;⚠️ &lt;b&gt;Could not add quote line item&lt;/b&gt;&lt;br/&gt;Missing parameter: QuoteId&lt;/div&gt;</t>
+          <t>Skill executed successfully (Apex business success).</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Enable Salesforce Quotes (Setup → Feature Settings → Sales → Quotes → Enable Quotes), create a seed Quote (with Pricebook and optional line items), then re-run.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1943,7 +1947,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>fail_missing_feature</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1953,22 +1957,22 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>{ "Name": "E2E Quote", "OpportunityId": "006QH00000Kz5M9YAJ" }</t>
+          <t>{ "Name": "E2E Quote 1137", "OpportunityId": "006QH00000Kz5M9YAJ" }</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>&lt;div&gt;⚠️ &lt;b&gt;Could not create quote&lt;/b&gt;&lt;br/&gt;Quote is not creatable (enable Quotes).&lt;/div&gt;</t>
+          <t>{ "status": "Success", "message": "", "data": { "recordId": "0Q0QH000002BnIn0AK", "message": "✅ Quote Created Name: E2E Quote 1137 👉 View Quote", "success": true } }</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Feature / package not available in this org (expected N/A until enabled).</t>
+          <t>Skill executed successfully (Apex business success).</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Enable Salesforce Quotes in Setup, then create at least one Quote (and Quote Line if testing line skills) on the E2E Opportunity/Account and re-run.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2789,7 +2793,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>fail_missing_feature</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2799,22 +2803,22 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>{ "Id": "001QH00002FpgehYAB" }</t>
+          <t>{ "Id": "ka0QH000000EUpRYAW", "Title": "Test 1" }</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Knowledge is not enabled in this org.</t>
+          <t>{ "status": "Success", "message": "", "data": { "success": true, "recordUrl": "https://masterdev4-dev-ed.develop.my.salesforce.com/lightning/r/Knowledge__kav/ka0QH000000EUpRYAW/view", "PublishStatus": "Online", "VersionNumber": 1, "UrlName": "Test-1", "ArticleNumber": "000001000", "Summary": null, "Title": "Test 1", "KnowledgeArticleId": "kA0QH000000BR9l0AG", "Id": "ka0QH000000EUpRYAW" } }</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Feature / package not available in this org (expected N/A until enabled).</t>
+          <t>Skill executed successfully (Apex business success).</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Enable Lightning Knowledge (Setup → Knowledge Settings), create a published article, assign Knowledge user permissions, then re-run.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -3118,7 +3122,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>fail_missing_feature</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -3128,22 +3132,22 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>{ "OpportunityId": "E2E Skill Test Opp", "OpportunityName": "E2E Skill Test Opp", "Id": "006QH00000Kz5M9YAJ" }</t>
+          <t>{ "OpportunityId": "006QH00000Kz5M9YAJ", "OpportunityName": "E2E Skill Test Opp", "Id": "006QH00000Kz5M9YAJ" }</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>OpportunityTeamMember is not accessible (Team Selling may be disabled).</t>
+          <t>{ "status": "Success", "message": "", "data": { "success": true, "teamMembers": [ { "recordUrl": "https://masterdev4-dev-ed.develop.my.salesforce.com/lightning/r/OpportunityTeamMember/00qQH000006mt0MYAQ/view", "TeamMemberRole": "Channel Manager", "UserName": "Kalanithi Balasubramanian", "UserId": "005QH00000Ahc4IYAR", "Id": "00qQH000006mt0MYAQ" } ], "count": 1, "OpportunityId": "006QH00000Kz5M9YAJ" } }</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Feature / package not available in this org (expected N/A until enabled).</t>
+          <t>Skill executed successfully (Apex business success).</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Enable Team Selling (Setup → Opportunity Team Settings / Team Selling), ensure OpportunityTeamMember is creatable, then re-run.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -3447,7 +3451,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>fail_missing_feature</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3457,22 +3461,22 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>{ "Id": "001QH00002FpgehYAB" }</t>
+          <t>{ "Id": "0Q0QH000002Bn7V0AS", "Name": "Quote 1" }</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Quote is not available or accessible in this org (enable Quotes).</t>
+          <t>{ "status": "Success", "message": "", "data": { "success": true, "recordUrl": "https://masterdev4-dev-ed.develop.my.salesforce.com/lightning/r/Quote/0Q0QH000002Bn7V0AS/view", "Pricebook2Id": "01sQH000004ETvuYAG", "Owner": "Kalanithi Balasubramanian", "Account": "E2E Skill Test Account", "Opportunity": "E2E Skill Test Opp", "Description": null, "ExpirationDate": "2026-08-17 00:00:00", "Discount": 0.0, "TotalPrice": 210.0, "Subtotal": 210.0, "GrandTotal": 210.0, "Status": "Draft", "QuoteNumber": "00000001", "Name": "Quote 1", "Id": "0Q0QH000002Bn7V0AS" } }</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Feature / package not available in this org (expected N/A until enabled).</t>
+          <t>Skill executed successfully (Apex business success).</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Enable Salesforce Quotes in Setup, then create at least one Quote (and Quote Line if testing line skills) on the E2E Opportunity/Account and re-run.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -4340,7 +4344,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>fail_missing_feature</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4350,22 +4354,22 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>{ "searchTerm": "Quote", "search_term": "Quote" }</t>
+          <t>{ "searchTerm": "Quote 1", "search_term": "Quote 1" }</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Quote is not available or accessible in this org (enable Quotes).</t>
+          <t>{ "status": "Success", "message": "", "data": { "success": true, "records": [ { "viewRecord": "&lt;a href=\"https://masterdev4-dev-ed.develop.my.salesforce.com/lightning/r/Quote/0Q0QH000002BnIn0AK/view\" target=\"_blank\"&gt;View Record&lt;/a&gt;", "recordUrl": "https://masterdev4-dev-ed.develop.my.salesforce.com/lightning/r/Quote/0Q0QH000002BnIn0AK/view", "OpportunityId": "006QH00000Kz5M9YAJ", "GrandTotal": 0.0, "Status": "Draft", "QuoteNumber": "00000002", "Name": "E2E Quote 1137", "Id": "0Q0QH000002BnIn0AK" }, { "viewRecord": "&lt;a href=\"https://masterdev4-dev-ed.develop.my.salesforce.com/lightning/r/Quote/0Q0QH000002Bn7V0AS/view\" target=\"_blank\"&gt;View Record&lt;/a&gt;", "recordUrl": "https://masterdev4-dev-ed.develop.my.salesforce.com/lightning/r/Quote/0Q0QH000002Bn7V0AS/view", "OpportunityId": "006QH00000Kz5M9YAJ", "GrandTotal": 210.0, "Status": "Draft", "QuoteNumber": "00000001", "Name": "Quote 1", "Id": "0Q0QH000002Bn7V0AS" } ], "remaining": 0, "displayed": 2, "totalFound": 2, "status": "found" } }</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Feature / package not available in this org (expected N/A until enabled).</t>
+          <t>Skill executed successfully (Apex business success).</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Enable Salesforce Quotes in Setup, then create at least one Quote (and Quote Line if testing line skills) on the E2E Opportunity/Account and re-run.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -4387,7 +4391,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>fail_missing_feature</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4397,22 +4401,22 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>{ "case_id": "500QH00000VaKnyYAF", "CaseId": "500QH00000VaKnyYAF", "KnowledgeArticleId": "500QH00000VaKnyYAF", "Id": "500QH00000VaKnyYAF" }</t>
+          <t>{ "case_id": "500QH00000VaKnyYAF", "CaseId": "500QH00000VaKnyYAF", "article_id": "ka0QH000000EUpRYAW", "KnowledgeArticleId": "kA0QH000000BR9l0AG", "Id": "ka0QH000000EUpRYAW" }</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>&lt;div&gt;⚠️ &lt;b&gt;Could not link article&lt;/b&gt;&lt;br/&gt;CaseArticle is not available in this org (Knowledge may not be enabled).&lt;/div&gt;</t>
+          <t>{ "status": "Success", "message": "", "data": { "recordId": "0gvQH0000001kjxYAA", "message": "✅ Knowledge Article Linked Case #: 00001037 Article linked 👉 View Link", "success": true } }</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Feature / package not available in this org (expected N/A until enabled).</t>
+          <t>Skill executed successfully (Apex business success).</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Enable Lightning Knowledge (Setup → Knowledge Settings), create a published article, assign Knowledge user permissions, then re-run.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -4622,7 +4626,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>fail_missing_feature</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -4632,22 +4636,22 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>{ "search_term": "test", "searchTerm": "test" }</t>
+          <t>{ "search_term": "Test 1", "searchTerm": "Test 1" }</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Knowledge is not enabled in this org.</t>
+          <t>{ "status": "Success", "message": "", "data": { "success": true, "articles": [ { "recordUrl": "https://masterdev4-dev-ed.develop.my.salesforce.com/lightning/r/Knowledge__kav/ka0QH000000EUpRYAW/view", "UrlName": "Test-1", "ArticleNumber": "000001000", "Summary": null, "Title": "Test 1", "KnowledgeArticleId": "kA0QH000000BR9l0AG", "Id": "ka0QH000000EUpRYAW" } ], "count": 1, "searchTerm": "Test 1" } }</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Feature / package not available in this org (expected N/A until enabled).</t>
+          <t>Skill executed successfully (Apex business success).</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Enable Lightning Knowledge (Setup → Knowledge Settings), create a published article, assign Knowledge user permissions, then re-run.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -5562,7 +5566,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>fail_data</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -5572,22 +5576,22 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>{ "Description": "E2E" }</t>
+          <t>{ "Id": "0Q0QH000002Bn7V0AS", "Description": "E2E quote update" }</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>&lt;div&gt;⚠️ &lt;b&gt;Could not update quote&lt;/b&gt;&lt;br/&gt;Missing parameter: quote_id&lt;/div&gt;</t>
+          <t>{ "status": "Success", "message": "", "data": { "recordId": "0Q0QH000002Bn7V0AS", "message": "✅ Quote Updated Quote 1 Description: (none) → E2E quote update 👉 View Quote", "success": true } }</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Data / seed or missing parameter issue: &lt;div&gt;⚠️ &lt;b&gt;Could not update quote&lt;/b&gt;&lt;br/&gt;Missing parameter: quote_id&lt;/div&gt;</t>
+          <t>Skill executed successfully (Apex business success).</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Enable Salesforce Quotes (Setup → Feature Settings → Sales → Quotes → Enable Quotes), create a seed Quote (with Pricebook and optional line items), then re-run.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -5609,7 +5613,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>fail_data</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -5619,22 +5623,22 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>{ "Quantity": 2 }</t>
+          <t>{ "Id": "0QLQH000003nalN4AQ", "Quantity": 2 }</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>&lt;div&gt;⚠️ &lt;b&gt;Could not update quote line item&lt;/b&gt;&lt;br/&gt;Missing parameter: line_item_id&lt;/div&gt;</t>
+          <t>{ "status": "Success", "message": "", "data": { "recordId": "0QLQH000003nalN4AQ", "message": "✅ Quote Line Item Updated Line item (2.00 @ 50.00) Quantity: 2.00 → 2.00 👉 View Line Item", "success": true } }</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Data / seed or missing parameter issue: &lt;div&gt;⚠️ &lt;b&gt;Could not update quote line item&lt;/b&gt;&lt;br/&gt;Missing parameter: line_item_id&lt;/div&gt;</t>
+          <t>Skill executed successfully (Apex business success).</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Enable Salesforce Quotes in Setup, then create at least one Quote (and Quote Line if testing line skills) on the E2E Opportunity/Account and re-run.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">

</xml_diff>